<commit_message>
new package structure - some tests checked
</commit_message>
<xml_diff>
--- a/tests/coil_2D_avolt_timint/input_template.xlsx
+++ b/tests/coil_2D_avolt_timint/input_template.xlsx
@@ -143,7 +143,7 @@
     <t>VARIABLE</t>
   </si>
   <si>
-    <t>V</t>
+    <t>VOLT</t>
   </si>
   <si>
     <t>TYPE_ID</t>
@@ -172,7 +172,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,6 +183,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -219,13 +225,13 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -234,7 +240,7 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -929,7 +935,7 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4">
         <v>1</v>
       </c>

</xml_diff>